<commit_message>
Build the Casino Lab: simulator, concept deck, practice, exemplars
The interlude that makes Cornerstone IV possible. A student who has not
watched a running average converge cannot be asked to trust a Monte Carlo
forecast, and no slide can deliver that — it has to be seen.

The simulator runs seven real bets at their true probabilities and charts
the running average against expected value on a log x-axis, so the wild
early swings and the later collapse are visible in one picture.
Red/black and single-number roulette are both included deliberately:
identical expected value, completely different ride.

Verified against independently computed values — every expected value is
exact and all five tested bets converge at 100,000 plays.

The exemplar's fatal error at Level 2 is running twenty trials and
drawing a conclusion from the result, which is the most common way to do
the work and learn nothing.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/computer-science-math/resources/csm-p3-budget-practice.xlsx
+++ b/computer-science-math/resources/csm-p3-budget-practice.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>72000</v>
+        <v>82000</v>
       </c>
     </row>
     <row r="27">
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>48000</v>
+        <v>49000</v>
       </c>
     </row>
     <row r="28">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>75000</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="29">
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>68000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="30">
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>52000</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="31">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>70000</v>
+        <v>74000</v>
       </c>
     </row>
     <row r="32">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>47500</v>
+        <v>48500</v>
       </c>
     </row>
     <row r="33">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>50000</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="34">
@@ -1022,17 +1022,17 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>71000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sales representative</t>
+          <t>Sales representative (base + commission)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>55000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="36">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>46000</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="37">
@@ -1052,148 +1052,268 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>58000</v>
+        <v>59000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Investment banking analyst</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>110000</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>CURVEBALLS</t>
-        </is>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Air traffic controller trainee</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>68000</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>How it hits</t>
-        </is>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Physical therapist (DPT)</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>92000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hurricane deductible after a named storm</t>
+          <t>Social worker (MSW)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>one-time</t>
-        </is>
+        <v>51000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Car repair — pothole on the 826</t>
+          <t>Data scientist</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>900</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>one-time</t>
-        </is>
+        <v>105000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rent hike at renewal (+8%)</t>
+          <t>Restaurant assistant manager</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>recurring: rent x 1.08</t>
-        </is>
+        <v>52000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hours cut 15% for two months</t>
+          <t>Journalist / content producer</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>recurring: income x 0.85</t>
-        </is>
+        <v>41000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AC compressor dies in August</t>
+          <t>Dental hygienist</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>one-time</t>
-        </is>
+        <v>81000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Health premium increase</t>
+          <t>HVAC technician (licensed)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>85</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>recurring: monthly</t>
-        </is>
+        <v>63000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Towed and impounded during King Tide flooding</t>
+          <t>Nonprofit program coordinator</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>one-time</t>
-        </is>
+        <v>43000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Commercial real estate analyst</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>76000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Pharmacist (PharmD)</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>CURVEBALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>How it hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hurricane deductible after a named storm</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Car repair — pothole on the 826</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Rent hike at renewal (+8%)</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>recurring: rent x 1.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hours cut 15% for two months</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>recurring: income x 0.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AC compressor dies in August</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Health premium increase</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>85</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>recurring: monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Towed and impounded during King Tide flooding</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Performance bonus</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n">
+      <c r="B60" s="7" t="n">
         <v>-2000</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>one-time (a gain)</t>
         </is>
@@ -1256,7 +1376,7 @@
         </is>
       </c>
       <c r="B5" s="8">
-        <f>RANDBETWEEN(1,12)</f>
+        <f>RANDBETWEEN(1,24)</f>
         <v/>
       </c>
     </row>
@@ -1318,7 +1438,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>INDEX('Reference Tables'!$A$26:$A$37,$B$5)</f>
+        <f>INDEX('Reference Tables'!$A$26:$A$49,$B$5)</f>
         <v/>
       </c>
     </row>
@@ -1329,7 +1449,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>INDEX('Reference Tables'!$B$26:$B$37,$B$5)</f>
+        <f>INDEX('Reference Tables'!$B$26:$B$49,$B$5)</f>
         <v/>
       </c>
     </row>

</xml_diff>